<commit_message>
Format dates, times, and durations; add xl_valid()
DateTime cells now render as 'YYYY-MM-DD' for date-only values,
'HH:MM:SS' for time-only values and durations, and a full datetime
otherwise. Regenerate test fixtures with real date/time/datetime
columns. Add xl_valid(blob) to check whether a blob is a readable
workbook.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/students.xlsx
+++ b/tests/students.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>id</t>
   </si>
@@ -30,6 +30,12 @@
     <t>email</t>
   </si>
   <si>
+    <t>enrollment_date</t>
+  </si>
+  <si>
+    <t>birth_date</t>
+  </si>
+  <si>
     <t>Alice Chen</t>
   </si>
   <si>
@@ -69,6 +75,9 @@
     <t>max_score</t>
   </si>
   <si>
+    <t>due_date</t>
+  </si>
+  <si>
     <t>Essay: Modern Poetry</t>
   </si>
   <si>
@@ -105,40 +114,18 @@
     <t>submitted</t>
   </si>
   <si>
-    <t>2025-03-10</t>
-  </si>
-  <si>
-    <t>2025-03-12</t>
-  </si>
-  <si>
-    <t>2025-03-15</t>
-  </si>
-  <si>
-    <t>2025-03-11</t>
-  </si>
-  <si>
-    <t>2025-03-14</t>
-  </si>
-  <si>
-    <t>2025-03-13</t>
-  </si>
-  <si>
-    <t>2025-03-18</t>
-  </si>
-  <si>
-    <t>2025-03-16</t>
-  </si>
-  <si>
-    <t>2025-03-17</t>
-  </si>
-  <si>
-    <t>2025-03-19</t>
+    <t>time_spent</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="hh:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -168,8 +155,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,10 +454,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -480,75 +470,111 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1">
+        <v>45159</v>
+      </c>
+      <c r="F2" s="1">
+        <v>39918</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>9</v>
+      </c>
+      <c r="E3" s="1">
+        <v>44795</v>
+      </c>
+      <c r="F3" s="1">
+        <v>39755</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1">
+        <v>45159</v>
+      </c>
+      <c r="F4" s="1">
+        <v>40022</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1">
+        <v>44431</v>
+      </c>
+      <c r="F5" s="1">
+        <v>39417</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="E6" s="1">
+        <v>44795</v>
+      </c>
+      <c r="F6" s="1">
+        <v>39618</v>
       </c>
     </row>
   </sheetData>
@@ -558,77 +584,92 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D2">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2" s="2">
+        <v>45730.99930555555</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D3">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3" s="2">
+        <v>45731.64583333334</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>75</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4" s="2">
+        <v>45734.99930555555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D5">
         <v>100</v>
+      </c>
+      <c r="E5" s="2">
+        <v>45736.375</v>
       </c>
     </row>
   </sheetData>
@@ -638,24 +679,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>31</v>
+      </c>
+      <c r="E1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -665,11 +709,14 @@
       <c r="C2">
         <v>92</v>
       </c>
-      <c r="D2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="D2" s="2">
+        <v>45726.60416666666</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.07291666666666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>1</v>
       </c>
@@ -679,11 +726,14 @@
       <c r="C3">
         <v>47</v>
       </c>
-      <c r="D3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="D3" s="2">
+        <v>45728.38541666666</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.03472222222222222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>1</v>
       </c>
@@ -693,11 +743,14 @@
       <c r="C4">
         <v>71</v>
       </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="D4" s="2">
+        <v>45731.91666666666</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.09027777777777778</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>2</v>
       </c>
@@ -707,11 +760,14 @@
       <c r="C5">
         <v>85</v>
       </c>
-      <c r="D5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="D5" s="2">
+        <v>45727.69791666666</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>2</v>
       </c>
@@ -721,11 +777,14 @@
       <c r="C6">
         <v>44</v>
       </c>
-      <c r="D6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="D6" s="2">
+        <v>45728.41666666666</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.02777777777777778</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>2</v>
       </c>
@@ -735,11 +794,14 @@
       <c r="C7">
         <v>68</v>
       </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="D7" s="2">
+        <v>45730.85416666666</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.0798611111111111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>3</v>
       </c>
@@ -749,11 +811,14 @@
       <c r="C8">
         <v>97</v>
       </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="D8" s="2">
+        <v>45726.33333333334</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.1041666666666667</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>3</v>
       </c>
@@ -763,11 +828,14 @@
       <c r="C9">
         <v>50</v>
       </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="D9" s="2">
+        <v>45729.58333333334</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.03125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>3</v>
       </c>
@@ -777,11 +845,14 @@
       <c r="C10">
         <v>88</v>
       </c>
-      <c r="D10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="D10" s="2">
+        <v>45734.47916666666</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0.05555555555555555</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>4</v>
       </c>
@@ -791,11 +862,14 @@
       <c r="C11">
         <v>78</v>
       </c>
-      <c r="D11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="D11" s="2">
+        <v>45727.79166666666</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0.05208333333333334</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12">
         <v>4</v>
       </c>
@@ -805,11 +879,14 @@
       <c r="C12">
         <v>72</v>
       </c>
-      <c r="D12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="D12" s="2">
+        <v>45732.90625</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0.08333333333333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13">
         <v>4</v>
       </c>
@@ -819,11 +896,14 @@
       <c r="C13">
         <v>95</v>
       </c>
-      <c r="D13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="D13" s="2">
+        <v>45733.42708333334</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0.07291666666666667</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14">
         <v>5</v>
       </c>
@@ -833,11 +913,14 @@
       <c r="C14">
         <v>41</v>
       </c>
-      <c r="D14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="D14" s="2">
+        <v>45728.47916666666</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.02430555555555556</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15">
         <v>5</v>
       </c>
@@ -847,11 +930,14 @@
       <c r="C15">
         <v>60</v>
       </c>
-      <c r="D15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="D15" s="2">
+        <v>45731.99652777778</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.06944444444444445</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16">
         <v>5</v>
       </c>
@@ -861,8 +947,11 @@
       <c r="C16">
         <v>82</v>
       </c>
-      <c r="D16" t="s">
-        <v>38</v>
+      <c r="D16" s="2">
+        <v>45735.36458333334</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.04861111111111111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>